<commit_message>
Updated Data Test Id Attribute Locators In Pom, Sales, PMF Modules
Updated Data Test Id Attribute Locators In Pom, Sales, PMF Modules
</commit_message>
<xml_diff>
--- a/testdata/ProductionCalculations.xlsx
+++ b/testdata/ProductionCalculations.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="ProductionWithResources" sheetId="1" r:id="rId1"/>
+    <sheet name="ProductionWithMultipleResources" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="24">
   <si>
     <t>Machine Cost</t>
   </si>
@@ -53,7 +54,34 @@
     <t>Line Amount</t>
   </si>
   <si>
-    <t>GWLPROCESS-01</t>
+    <t>Line Amount UC</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>Employee Name</t>
+  </si>
+  <si>
+    <t>Qty Hrs</t>
+  </si>
+  <si>
+    <t>Raw Material Cost</t>
+  </si>
+  <si>
+    <t>RM UC</t>
+  </si>
+  <si>
+    <t>Qty</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>UnitCost</t>
+  </si>
+  <si>
+    <t>GWLPROCESS-02</t>
   </si>
   <si>
     <t>GWLMACHINE</t>
@@ -62,41 +90,30 @@
     <t>GWL MACHINE 1</t>
   </si>
   <si>
-    <t>GWLPROCESS-02</t>
-  </si>
-  <si>
-    <t>Labour Cost</t>
-  </si>
-  <si>
-    <t>SNO</t>
-  </si>
-  <si>
-    <t>Employee</t>
-  </si>
-  <si>
-    <t>Employee Name</t>
-  </si>
-  <si>
-    <t>Qty Hrs</t>
-  </si>
-  <si>
     <t>TVS00355</t>
   </si>
   <si>
     <t>GWL MAN 1</t>
+  </si>
+  <si>
+    <t>210.00</t>
+  </si>
+  <si>
+    <t>GWLPROCESS-03</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="180" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,14 +143,6 @@
       <name val="Calibri Light"/>
       <charset val="134"/>
       <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -632,137 +641,137 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -787,15 +796,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="180" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -855,13 +859,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
-<customStorage xmlns="https://web.wps.cn/et/2018/main">
-  <book/>
-  <sheets/>
-</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1122,8 +1119,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="6"/>
+  <dimension ref="A1:S7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="6"/>
   <cols>
     <col min="1" max="1" width="6.77777777777778" style="1" customWidth="1"/>
     <col min="2" max="2" width="15" style="1" customWidth="1"/>
@@ -1131,9 +1128,17 @@
     <col min="4" max="4" width="29.2222222222222" customWidth="1"/>
     <col min="5" max="6" width="10.1111111111111" customWidth="1"/>
     <col min="7" max="7" width="13.4444444444444" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="13.4444444444444" customWidth="1"/>
+    <col min="10" max="10" width="16.8888888888889" customWidth="1"/>
+    <col min="11" max="13" width="13.4444444444444" customWidth="1"/>
+    <col min="14" max="15" width="19.1111111111111" customWidth="1"/>
+    <col min="16" max="16" width="7.77777777777778" customWidth="1"/>
+    <col min="17" max="18" width="6.22222222222222" customWidth="1"/>
+    <col min="19" max="19" width="12.8888888888889"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.6" spans="1:7">
+    <row r="1" ht="15.6" spans="1:13">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1143,8 +1148,14 @@
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
     </row>
-    <row r="2" ht="15.15" spans="1:7">
+    <row r="2" ht="15.15" spans="1:19">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1166,19 +1177,55 @@
       <c r="G2" s="5" t="s">
         <v>7</v>
       </c>
+      <c r="H2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="3" ht="15.15" spans="1:7">
+    <row r="3" ht="15.15" spans="1:19">
       <c r="A3" s="6">
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E3" s="7">
         <v>9.5</v>
@@ -1190,19 +1237,61 @@
         <f>E3*F3</f>
         <v>399</v>
       </c>
+      <c r="H3" s="7">
+        <f>G3/Q3</f>
+        <v>133</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="7">
+        <v>9.5</v>
+      </c>
+      <c r="L3" s="7">
+        <v>100</v>
+      </c>
+      <c r="M3" s="6">
+        <f>K3*L3</f>
+        <v>950</v>
+      </c>
+      <c r="N3" s="11">
+        <f>M3/Q3</f>
+        <v>316.666666666667</v>
+      </c>
+      <c r="O3" t="s">
+        <v>22</v>
+      </c>
+      <c r="P3" s="7">
+        <f>O3/Q3</f>
+        <v>70</v>
+      </c>
+      <c r="Q3" s="7">
+        <v>3</v>
+      </c>
+      <c r="R3" s="7">
+        <f>(G3+O3+M3)</f>
+        <v>1419</v>
+      </c>
+      <c r="S3" s="11">
+        <f>H3+N3+P3</f>
+        <v>519.666666666667</v>
+      </c>
     </row>
-    <row r="4" ht="15.15" spans="1:7">
+    <row r="4" ht="15.15" spans="1:19">
       <c r="A4" s="6">
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E4" s="7">
         <v>9.5</v>
@@ -1211,11 +1300,53 @@
         <v>42</v>
       </c>
       <c r="G4" s="7">
-        <f t="shared" ref="G4:G9" si="0">E4*F4</f>
+        <f>E4*F4</f>
         <v>399</v>
       </c>
+      <c r="H4" s="7">
+        <f>G4/Q4</f>
+        <v>133</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="7">
+        <v>9.5</v>
+      </c>
+      <c r="L4" s="7">
+        <v>100</v>
+      </c>
+      <c r="M4" s="6">
+        <f>K4*L4</f>
+        <v>950</v>
+      </c>
+      <c r="N4" s="11">
+        <f>M4/Q4</f>
+        <v>316.666666666667</v>
+      </c>
+      <c r="O4" s="7">
+        <v>140</v>
+      </c>
+      <c r="P4" s="7">
+        <f>O4/Q4</f>
+        <v>46.6666666666667</v>
+      </c>
+      <c r="Q4" s="7">
+        <v>3</v>
+      </c>
+      <c r="R4" s="7">
+        <f>(G4+O4+M4)</f>
+        <v>1489</v>
+      </c>
+      <c r="S4" s="11">
+        <f>H4+N4+P4</f>
+        <v>496.333333333333</v>
+      </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:13">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="9"/>
@@ -1223,96 +1354,335 @@
       <c r="E5" s="9"/>
       <c r="F5" s="9"/>
       <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
-    <row r="6" ht="18" spans="1:7">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="3:3">
+      <c r="C6" s="10"/>
+    </row>
+    <row r="7" spans="1:19">
+      <c r="A7" s="1">
+        <v>0</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7">
+        <v>4</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7">
+        <v>6</v>
+      </c>
+      <c r="H7">
+        <v>7</v>
+      </c>
+      <c r="I7">
+        <v>8</v>
+      </c>
+      <c r="J7">
+        <v>9</v>
+      </c>
+      <c r="K7">
+        <v>10</v>
+      </c>
+      <c r="L7">
+        <v>11</v>
+      </c>
+      <c r="M7">
         <v>12</v>
       </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-    </row>
-    <row r="7" ht="15.15" spans="1:7">
-      <c r="A7" s="4" t="s">
+      <c r="N7">
         <v>13</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="O7">
         <v>14</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="P7">
         <v>15</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="Q7">
         <v>16</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" ht="15.15" spans="1:7">
-      <c r="A8" s="6">
-        <v>1</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="7" t="s">
+      <c r="R7">
         <v>17</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="S7">
         <v>18</v>
       </c>
-      <c r="E8" s="7">
-        <v>9.5</v>
-      </c>
-      <c r="F8" s="7">
-        <v>100</v>
-      </c>
-      <c r="G8" s="7">
-        <f t="shared" si="0"/>
-        <v>950</v>
-      </c>
-    </row>
-    <row r="9" ht="15.15" spans="1:7">
-      <c r="A9" s="6">
-        <v>1</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" s="7">
-        <v>9.5</v>
-      </c>
-      <c r="F9" s="7">
-        <v>100</v>
-      </c>
-      <c r="G9" s="7">
-        <f t="shared" si="0"/>
-        <v>950</v>
-      </c>
-    </row>
-    <row r="12" spans="3:3">
-      <c r="C12" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A6:G6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:S6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
+  <cols>
+    <col min="1" max="1" width="6.77777777777778" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.2222222222222" customWidth="1"/>
+    <col min="4" max="4" width="29.2222222222222" customWidth="1"/>
+    <col min="5" max="6" width="10.1111111111111" customWidth="1"/>
+    <col min="7" max="7" width="13.4444444444444" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="13.4444444444444" customWidth="1"/>
+    <col min="10" max="10" width="16.8888888888889" customWidth="1"/>
+    <col min="11" max="13" width="13.4444444444444" customWidth="1"/>
+    <col min="14" max="15" width="19.1111111111111" customWidth="1"/>
+    <col min="16" max="16" width="7.77777777777778" customWidth="1"/>
+    <col min="17" max="18" width="6.22222222222222" customWidth="1"/>
+    <col min="19" max="19" width="12.8888888888889"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15.6" spans="1:13">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+    </row>
+    <row r="2" ht="15.15" spans="1:19">
+      <c r="A2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
+      <c r="A3" s="6">
+        <v>1</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="7">
+        <v>9.5</v>
+      </c>
+      <c r="F3" s="7">
+        <v>42</v>
+      </c>
+      <c r="G3" s="7">
+        <f>E3*F3</f>
+        <v>399</v>
+      </c>
+      <c r="H3" s="7">
+        <f>G3/Q3</f>
+        <v>133</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="7">
+        <v>9.5</v>
+      </c>
+      <c r="L3" s="7">
+        <v>100</v>
+      </c>
+      <c r="M3" s="6">
+        <f>K3*L3</f>
+        <v>950</v>
+      </c>
+      <c r="N3" s="11">
+        <f>M3/Q3</f>
+        <v>316.666666666667</v>
+      </c>
+      <c r="O3">
+        <v>210</v>
+      </c>
+      <c r="P3" s="7">
+        <f>O3/Q3</f>
+        <v>70</v>
+      </c>
+      <c r="Q3" s="7">
+        <v>3</v>
+      </c>
+      <c r="R3" s="7">
+        <f>(G3+O3+M3)</f>
+        <v>1559</v>
+      </c>
+      <c r="S3" s="11">
+        <f>H3+N3+P3</f>
+        <v>519.666666666667</v>
+      </c>
+    </row>
+    <row r="4" ht="15.15" spans="1:19">
+      <c r="A4" s="6">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="7">
+        <v>9.5</v>
+      </c>
+      <c r="F4" s="7">
+        <v>42</v>
+      </c>
+      <c r="G4" s="7">
+        <f>E4*F4</f>
+        <v>399</v>
+      </c>
+      <c r="H4" s="7">
+        <f>G4/Q4</f>
+        <v>133</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="7">
+        <v>9.5</v>
+      </c>
+      <c r="L4" s="7">
+        <v>100</v>
+      </c>
+      <c r="M4" s="6">
+        <f>K4*L4</f>
+        <v>950</v>
+      </c>
+      <c r="N4" s="11">
+        <f>M4/Q4</f>
+        <v>316.666666666667</v>
+      </c>
+      <c r="O4" s="7">
+        <v>140</v>
+      </c>
+      <c r="P4" s="7">
+        <f>O4/Q4</f>
+        <v>46.6666666666667</v>
+      </c>
+      <c r="Q4" s="7">
+        <v>3</v>
+      </c>
+      <c r="R4" s="7">
+        <f>(G4+O4+M4)</f>
+        <v>1489</v>
+      </c>
+      <c r="S4" s="11">
+        <f>H4+N4+P4</f>
+        <v>496.333333333333</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" spans="3:3">
+      <c r="C6" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>